<commit_message>
SPM-38: Record review test run (13 pass)
</commit_message>
<xml_diff>
--- a/docs/test-cases/SPM-38_Test_Cases.xlsx
+++ b/docs/test-cases/SPM-38_Test_Cases.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11020"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\IS212\docs\test-cases\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/janelleip/Documents/GitHub/IS212/docs/test-cases/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{68E3C490-A0E2-4A63-9593-3C53C8319E11}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{101EF0EC-34A1-974A-A9C3-A496BBCA725B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9510" yWindow="0" windowWidth="9780" windowHeight="10170" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="15980" activeTab="14" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" r:id="rId1"/>
@@ -29,12 +29,25 @@
     <sheet name="TC12" sheetId="14" r:id="rId14"/>
     <sheet name="TC13" sheetId="15" r:id="rId15"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="501" uniqueCount="179">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="670" uniqueCount="182">
   <si>
     <t>Story</t>
   </si>
@@ -827,6 +840,15 @@
   </si>
   <si>
     <t>Kayalvizhi</t>
+  </si>
+  <si>
+    <t>6c0c6eb</t>
+  </si>
+  <si>
+    <t>Janelle</t>
+  </si>
+  <si>
+    <t>d1f2c08</t>
   </si>
 </sst>
 </file>
@@ -848,28 +870,33 @@
       <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
       <sz val="10"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <u/>
       <sz val="10"/>
       <color rgb="FF1155CC"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="5">
@@ -992,11 +1019,11 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1213,7 +1240,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:I29"/>
-  <sheetFormatPr defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="13" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="20" customWidth="1"/>
@@ -1226,22 +1253,22 @@
     <col min="9" max="9" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="31" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" ht="31" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="16" t="s">
+      <c r="B1" s="15" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="14"/>
-      <c r="D1" s="14"/>
-      <c r="E1" s="14"/>
-      <c r="F1" s="14"/>
-      <c r="G1" s="14"/>
-      <c r="H1" s="14"/>
-      <c r="I1" s="15"/>
-    </row>
-    <row r="3" spans="1:9" ht="13" x14ac:dyDescent="0.25">
+      <c r="C1" s="16"/>
+      <c r="D1" s="16"/>
+      <c r="E1" s="16"/>
+      <c r="F1" s="16"/>
+      <c r="G1" s="16"/>
+      <c r="H1" s="16"/>
+      <c r="I1" s="14"/>
+    </row>
+    <row r="3" spans="1:9" ht="14" x14ac:dyDescent="0.15">
       <c r="A3" s="7" t="s">
         <v>2</v>
       </c>
@@ -1270,7 +1297,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:9" ht="50" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" ht="56" x14ac:dyDescent="0.15">
       <c r="A4" s="8" t="s">
         <v>11</v>
       </c>
@@ -1295,7 +1322,7 @@
       <c r="H4" s="9"/>
       <c r="I4" s="9"/>
     </row>
-    <row r="5" spans="1:9" ht="50" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" ht="56" x14ac:dyDescent="0.15">
       <c r="A5" s="8" t="s">
         <v>18</v>
       </c>
@@ -1320,7 +1347,7 @@
       <c r="H5" s="9"/>
       <c r="I5" s="9"/>
     </row>
-    <row r="6" spans="1:9" ht="25" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" ht="28" x14ac:dyDescent="0.15">
       <c r="A6" s="8" t="s">
         <v>22</v>
       </c>
@@ -1345,7 +1372,7 @@
       <c r="H6" s="9"/>
       <c r="I6" s="9"/>
     </row>
-    <row r="7" spans="1:9" ht="37.5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" ht="42" x14ac:dyDescent="0.15">
       <c r="A7" s="8" t="s">
         <v>26</v>
       </c>
@@ -1370,7 +1397,7 @@
       <c r="H7" s="9"/>
       <c r="I7" s="9"/>
     </row>
-    <row r="8" spans="1:9" ht="37.5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" ht="42" x14ac:dyDescent="0.15">
       <c r="A8" s="8" t="s">
         <v>30</v>
       </c>
@@ -1395,7 +1422,7 @@
       <c r="H8" s="9"/>
       <c r="I8" s="9"/>
     </row>
-    <row r="9" spans="1:9" ht="37.5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" ht="42" x14ac:dyDescent="0.15">
       <c r="A9" s="8" t="s">
         <v>33</v>
       </c>
@@ -1420,7 +1447,7 @@
       <c r="H9" s="9"/>
       <c r="I9" s="9"/>
     </row>
-    <row r="10" spans="1:9" ht="50" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:9" ht="56" x14ac:dyDescent="0.15">
       <c r="A10" s="8" t="s">
         <v>37</v>
       </c>
@@ -1445,7 +1472,7 @@
       <c r="H10" s="9"/>
       <c r="I10" s="9"/>
     </row>
-    <row r="11" spans="1:9" ht="50" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9" ht="56" x14ac:dyDescent="0.15">
       <c r="A11" s="8" t="s">
         <v>41</v>
       </c>
@@ -1470,7 +1497,7 @@
       <c r="H11" s="9"/>
       <c r="I11" s="9"/>
     </row>
-    <row r="12" spans="1:9" ht="25" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:9" ht="28" x14ac:dyDescent="0.15">
       <c r="A12" s="8" t="s">
         <v>46</v>
       </c>
@@ -1495,7 +1522,7 @@
       <c r="H12" s="9"/>
       <c r="I12" s="9"/>
     </row>
-    <row r="13" spans="1:9" ht="37.5" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:9" ht="42" x14ac:dyDescent="0.15">
       <c r="A13" s="8" t="s">
         <v>51</v>
       </c>
@@ -1520,7 +1547,7 @@
       <c r="H13" s="9"/>
       <c r="I13" s="9"/>
     </row>
-    <row r="14" spans="1:9" ht="50" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:9" ht="56" x14ac:dyDescent="0.15">
       <c r="A14" s="8" t="s">
         <v>55</v>
       </c>
@@ -1545,7 +1572,7 @@
       <c r="H14" s="9"/>
       <c r="I14" s="9"/>
     </row>
-    <row r="15" spans="1:9" ht="37.5" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:9" ht="42" x14ac:dyDescent="0.15">
       <c r="A15" s="8" t="s">
         <v>59</v>
       </c>
@@ -1570,7 +1597,7 @@
       <c r="H15" s="9"/>
       <c r="I15" s="9"/>
     </row>
-    <row r="16" spans="1:9" ht="50" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:9" ht="42" x14ac:dyDescent="0.15">
       <c r="A16" s="8" t="s">
         <v>63</v>
       </c>
@@ -1595,150 +1622,149 @@
       <c r="H16" s="9"/>
       <c r="I16" s="9"/>
     </row>
-    <row r="19" spans="1:9" ht="13" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:9" ht="14" x14ac:dyDescent="0.15">
       <c r="A19" s="7" t="s">
         <v>67</v>
       </c>
-      <c r="B19" s="16" t="s">
+      <c r="B19" s="15" t="s">
         <v>68</v>
       </c>
-      <c r="C19" s="14"/>
-      <c r="D19" s="15"/>
-      <c r="E19" s="16" t="s">
+      <c r="C19" s="16"/>
+      <c r="D19" s="14"/>
+      <c r="E19" s="15" t="s">
         <v>69</v>
       </c>
-      <c r="F19" s="15"/>
-    </row>
-    <row r="20" spans="1:9" ht="112" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F19" s="14"/>
+    </row>
+    <row r="20" spans="1:9" ht="112" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A20" s="9" t="s">
         <v>49</v>
       </c>
       <c r="B20" s="13" t="s">
         <v>70</v>
       </c>
-      <c r="C20" s="14"/>
-      <c r="D20" s="15"/>
+      <c r="C20" s="16"/>
+      <c r="D20" s="14"/>
       <c r="E20" s="13" t="s">
         <v>71</v>
       </c>
-      <c r="F20" s="15"/>
-    </row>
-    <row r="21" spans="1:9" ht="44.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F20" s="14"/>
+    </row>
+    <row r="21" spans="1:9" ht="44.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A21" s="9" t="s">
         <v>58</v>
       </c>
       <c r="B21" s="13" t="s">
         <v>72</v>
       </c>
-      <c r="C21" s="14"/>
-      <c r="D21" s="15"/>
+      <c r="C21" s="16"/>
+      <c r="D21" s="14"/>
       <c r="E21" s="13" t="s">
         <v>73</v>
       </c>
-      <c r="F21" s="15"/>
-    </row>
-    <row r="22" spans="1:9" ht="44.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F21" s="14"/>
+    </row>
+    <row r="22" spans="1:9" ht="44.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A22" s="9" t="s">
         <v>21</v>
       </c>
       <c r="B22" s="13" t="s">
         <v>74</v>
       </c>
-      <c r="C22" s="14"/>
-      <c r="D22" s="15"/>
+      <c r="C22" s="16"/>
+      <c r="D22" s="14"/>
       <c r="E22" s="13" t="s">
         <v>75</v>
       </c>
-      <c r="F22" s="15"/>
-    </row>
-    <row r="23" spans="1:9" ht="44.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F22" s="14"/>
+    </row>
+    <row r="23" spans="1:9" ht="44.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A23" s="9" t="s">
         <v>76</v>
       </c>
       <c r="B23" s="13" t="s">
         <v>77</v>
       </c>
-      <c r="C23" s="14"/>
-      <c r="D23" s="15"/>
+      <c r="C23" s="16"/>
+      <c r="D23" s="14"/>
       <c r="E23" s="13" t="s">
         <v>78</v>
       </c>
-      <c r="F23" s="15"/>
-    </row>
-    <row r="24" spans="1:9" ht="44.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F23" s="14"/>
+    </row>
+    <row r="24" spans="1:9" ht="44.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A24" s="9" t="s">
         <v>79</v>
       </c>
       <c r="B24" s="13" t="s">
         <v>80</v>
       </c>
-      <c r="C24" s="14"/>
-      <c r="D24" s="15"/>
+      <c r="C24" s="16"/>
+      <c r="D24" s="14"/>
       <c r="E24" s="13" t="s">
         <v>81</v>
       </c>
-      <c r="F24" s="15"/>
-    </row>
-    <row r="25" spans="1:9" ht="44.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F24" s="14"/>
+    </row>
+    <row r="25" spans="1:9" ht="44.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A25" s="9" t="s">
         <v>62</v>
       </c>
       <c r="B25" s="13" t="s">
         <v>82</v>
       </c>
-      <c r="C25" s="14"/>
-      <c r="D25" s="15"/>
+      <c r="C25" s="16"/>
+      <c r="D25" s="14"/>
       <c r="E25" s="13" t="s">
         <v>83</v>
       </c>
-      <c r="F25" s="15"/>
-    </row>
-    <row r="26" spans="1:9" ht="71.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F25" s="14"/>
+    </row>
+    <row r="26" spans="1:9" ht="71.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A26" s="9" t="s">
         <v>84</v>
       </c>
       <c r="B26" s="13" t="s">
         <v>85</v>
       </c>
-      <c r="C26" s="14"/>
-      <c r="D26" s="15"/>
+      <c r="C26" s="16"/>
+      <c r="D26" s="14"/>
       <c r="E26" s="13" t="s">
         <v>64</v>
       </c>
-      <c r="F26" s="15"/>
-    </row>
-    <row r="27" spans="1:9" ht="31" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F26" s="14"/>
+    </row>
+    <row r="27" spans="1:9" ht="31" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A27" s="9" t="s">
         <v>86</v>
       </c>
       <c r="B27" s="13" t="s">
         <v>87</v>
       </c>
-      <c r="C27" s="14"/>
-      <c r="D27" s="15"/>
+      <c r="C27" s="16"/>
+      <c r="D27" s="14"/>
       <c r="E27" s="13" t="s">
         <v>38</v>
       </c>
-      <c r="F27" s="15"/>
-    </row>
-    <row r="29" spans="1:9" ht="233.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F27" s="14"/>
+    </row>
+    <row r="29" spans="1:9" ht="233.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A29" s="7" t="s">
         <v>88</v>
       </c>
       <c r="B29" s="13" t="s">
         <v>89</v>
       </c>
-      <c r="C29" s="14"/>
-      <c r="D29" s="14"/>
-      <c r="E29" s="14"/>
-      <c r="F29" s="14"/>
-      <c r="G29" s="14"/>
-      <c r="H29" s="14"/>
-      <c r="I29" s="15"/>
+      <c r="C29" s="16"/>
+      <c r="D29" s="16"/>
+      <c r="E29" s="16"/>
+      <c r="F29" s="16"/>
+      <c r="G29" s="16"/>
+      <c r="H29" s="16"/>
+      <c r="I29" s="14"/>
     </row>
   </sheetData>
   <mergeCells count="20">
-    <mergeCell ref="B1:I1"/>
     <mergeCell ref="B24:D24"/>
     <mergeCell ref="B20:D20"/>
     <mergeCell ref="B29:I29"/>
@@ -1758,6 +1784,7 @@
     <mergeCell ref="E20:F20"/>
     <mergeCell ref="B19:D19"/>
     <mergeCell ref="E19:F19"/>
+    <mergeCell ref="B1:I1"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="A4" location="'TC01'!A1" display="TC01" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
@@ -1783,20 +1810,20 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
-  <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:C25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
   <cols>
-    <col min="1" max="1" width="24.81640625" customWidth="1"/>
-    <col min="2" max="2" width="56.81640625" customWidth="1"/>
+    <col min="1" max="1" width="24.83203125" customWidth="1"/>
+    <col min="2" max="2" width="56.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="13" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" ht="13" x14ac:dyDescent="0.15">
       <c r="A1" s="1" t="s">
         <v>109</v>
       </c>
       <c r="B1" s="2"/>
     </row>
-    <row r="2" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A2" s="10" t="s">
         <v>3</v>
       </c>
@@ -1804,7 +1831,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="44.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" ht="44.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A3" s="10" t="s">
         <v>110</v>
       </c>
@@ -1812,7 +1839,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" ht="85" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A4" s="10" t="s">
         <v>111</v>
       </c>
@@ -1820,7 +1847,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="139" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" ht="139" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A5" s="10" t="s">
         <v>113</v>
       </c>
@@ -1828,7 +1855,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="58" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" ht="58" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A6" s="10" t="s">
         <v>115</v>
       </c>
@@ -1836,7 +1863,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="193" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" ht="193" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A7" s="10" t="s">
         <v>117</v>
       </c>
@@ -1844,7 +1871,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A8" s="10" t="s">
         <v>119</v>
       </c>
@@ -1852,7 +1879,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" ht="13" x14ac:dyDescent="0.15">
       <c r="A9" s="10" t="s">
         <v>121</v>
       </c>
@@ -1860,14 +1887,14 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="13" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" ht="13" x14ac:dyDescent="0.15">
       <c r="A11" s="4" t="s">
         <v>109</v>
       </c>
       <c r="B11" s="5"/>
       <c r="C11" s="6"/>
     </row>
-    <row r="12" spans="1:3" ht="175" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" ht="196" x14ac:dyDescent="0.15">
       <c r="A12" s="3" t="s">
         <v>122</v>
       </c>
@@ -1875,7 +1902,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" ht="13" x14ac:dyDescent="0.15">
       <c r="A13" s="3" t="s">
         <v>123</v>
       </c>
@@ -1883,7 +1910,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" ht="13" x14ac:dyDescent="0.15">
       <c r="A14" s="3" t="s">
         <v>124</v>
       </c>
@@ -1891,7 +1918,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" ht="13" x14ac:dyDescent="0.15">
       <c r="A15" s="3" t="s">
         <v>125</v>
       </c>
@@ -1899,7 +1926,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" ht="13" x14ac:dyDescent="0.15">
       <c r="A16" s="3" t="s">
         <v>126</v>
       </c>
@@ -1907,14 +1934,66 @@
         <v>46322</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" ht="13" x14ac:dyDescent="0.15">
       <c r="A17" s="3" t="s">
         <v>127</v>
       </c>
-      <c r="B17" s="3" t="inlineStr">
-        <is>
-          <t>6c0c6eb</t>
-        </is>
+      <c r="B17" s="3" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A19" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="B19" s="5"/>
+    </row>
+    <row r="20" spans="1:2" ht="198" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A20" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="B20" s="11" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A21" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A22" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="B22" s="3" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A23" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="B23" s="3" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A24" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="B24" s="12">
+        <v>46323</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A25" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="B25" s="3" t="s">
+        <v>181</v>
       </c>
     </row>
   </sheetData>
@@ -1927,20 +2006,20 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
-  <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:C25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
   <cols>
-    <col min="1" max="1" width="24.81640625" customWidth="1"/>
-    <col min="2" max="2" width="56.81640625" customWidth="1"/>
+    <col min="1" max="1" width="24.83203125" customWidth="1"/>
+    <col min="2" max="2" width="56.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="13" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" ht="13" x14ac:dyDescent="0.15">
       <c r="A1" s="1" t="s">
         <v>109</v>
       </c>
       <c r="B1" s="2"/>
     </row>
-    <row r="2" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A2" s="10" t="s">
         <v>3</v>
       </c>
@@ -1948,7 +2027,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="31" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" ht="31" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A3" s="10" t="s">
         <v>110</v>
       </c>
@@ -1956,7 +2035,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="125.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" ht="125.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A4" s="10" t="s">
         <v>111</v>
       </c>
@@ -1964,7 +2043,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="98.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" ht="98.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A5" s="10" t="s">
         <v>113</v>
       </c>
@@ -1972,7 +2051,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="58" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" ht="58" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A6" s="10" t="s">
         <v>115</v>
       </c>
@@ -1980,7 +2059,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" ht="85" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A7" s="10" t="s">
         <v>117</v>
       </c>
@@ -1988,7 +2067,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A8" s="10" t="s">
         <v>119</v>
       </c>
@@ -1996,7 +2075,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" ht="13" x14ac:dyDescent="0.15">
       <c r="A9" s="10" t="s">
         <v>121</v>
       </c>
@@ -2004,14 +2083,14 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="13" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" ht="13" x14ac:dyDescent="0.15">
       <c r="A11" s="4" t="s">
         <v>109</v>
       </c>
       <c r="B11" s="5"/>
       <c r="C11" s="6"/>
     </row>
-    <row r="12" spans="1:3" ht="75" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" ht="84" x14ac:dyDescent="0.15">
       <c r="A12" s="3" t="s">
         <v>122</v>
       </c>
@@ -2019,7 +2098,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" ht="13" x14ac:dyDescent="0.15">
       <c r="A13" s="3" t="s">
         <v>123</v>
       </c>
@@ -2027,7 +2106,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" ht="13" x14ac:dyDescent="0.15">
       <c r="A14" s="3" t="s">
         <v>124</v>
       </c>
@@ -2035,7 +2114,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" ht="13" x14ac:dyDescent="0.15">
       <c r="A15" s="3" t="s">
         <v>125</v>
       </c>
@@ -2043,7 +2122,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" ht="13" x14ac:dyDescent="0.15">
       <c r="A16" s="3" t="s">
         <v>126</v>
       </c>
@@ -2051,14 +2130,66 @@
         <v>46322</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" ht="13" x14ac:dyDescent="0.15">
       <c r="A17" s="3" t="s">
         <v>127</v>
       </c>
-      <c r="B17" s="3" t="inlineStr">
-        <is>
-          <t>6c0c6eb</t>
-        </is>
+      <c r="B17" s="3" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A19" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="B19" s="5"/>
+    </row>
+    <row r="20" spans="1:2" ht="100" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A20" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="B20" s="11" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A21" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A22" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="B22" s="3" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A23" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="B23" s="3" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A24" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="B24" s="12">
+        <v>46323</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A25" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="B25" s="3" t="s">
+        <v>181</v>
       </c>
     </row>
   </sheetData>
@@ -2071,20 +2202,20 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
-  <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:C25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
   <cols>
-    <col min="1" max="1" width="24.81640625" customWidth="1"/>
-    <col min="2" max="2" width="56.81640625" customWidth="1"/>
+    <col min="1" max="1" width="24.83203125" customWidth="1"/>
+    <col min="2" max="2" width="56.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="13" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" ht="13" x14ac:dyDescent="0.15">
       <c r="A1" s="1" t="s">
         <v>109</v>
       </c>
       <c r="B1" s="2"/>
     </row>
-    <row r="2" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A2" s="10" t="s">
         <v>3</v>
       </c>
@@ -2092,7 +2223,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="44.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" ht="44.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A3" s="10" t="s">
         <v>110</v>
       </c>
@@ -2100,7 +2231,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="98.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" ht="98.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A4" s="10" t="s">
         <v>111</v>
       </c>
@@ -2108,7 +2239,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="71.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" ht="71.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A5" s="10" t="s">
         <v>113</v>
       </c>
@@ -2116,7 +2247,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="58" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" ht="58" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A6" s="10" t="s">
         <v>115</v>
       </c>
@@ -2124,7 +2255,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="206.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" ht="206.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A7" s="10" t="s">
         <v>117</v>
       </c>
@@ -2132,7 +2263,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A8" s="10" t="s">
         <v>119</v>
       </c>
@@ -2140,7 +2271,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" ht="13" x14ac:dyDescent="0.15">
       <c r="A9" s="10" t="s">
         <v>121</v>
       </c>
@@ -2148,14 +2279,14 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="13" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" ht="13" x14ac:dyDescent="0.15">
       <c r="A11" s="4" t="s">
         <v>109</v>
       </c>
       <c r="B11" s="5"/>
       <c r="C11" s="6"/>
     </row>
-    <row r="12" spans="1:3" ht="175" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" ht="196" x14ac:dyDescent="0.15">
       <c r="A12" s="3" t="s">
         <v>122</v>
       </c>
@@ -2163,7 +2294,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" ht="13" x14ac:dyDescent="0.15">
       <c r="A13" s="3" t="s">
         <v>123</v>
       </c>
@@ -2171,7 +2302,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" ht="13" x14ac:dyDescent="0.15">
       <c r="A14" s="3" t="s">
         <v>124</v>
       </c>
@@ -2179,7 +2310,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" ht="13" x14ac:dyDescent="0.15">
       <c r="A15" s="3" t="s">
         <v>125</v>
       </c>
@@ -2187,7 +2318,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" ht="13" x14ac:dyDescent="0.15">
       <c r="A16" s="3" t="s">
         <v>126</v>
       </c>
@@ -2195,14 +2326,66 @@
         <v>46322</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" ht="13" x14ac:dyDescent="0.15">
       <c r="A17" s="3" t="s">
         <v>127</v>
       </c>
-      <c r="B17" s="3" t="inlineStr">
-        <is>
-          <t>6c0c6eb</t>
-        </is>
+      <c r="B17" s="3" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A19" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="B19" s="5"/>
+    </row>
+    <row r="20" spans="1:2" ht="199" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A20" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="B20" s="11" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A21" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A22" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="B22" s="3" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A23" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="B23" s="3" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A24" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="B24" s="12">
+        <v>46323</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A25" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="B25" s="3" t="s">
+        <v>181</v>
       </c>
     </row>
   </sheetData>
@@ -2215,20 +2398,20 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
-  <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:C25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
   <cols>
-    <col min="1" max="1" width="24.81640625" customWidth="1"/>
-    <col min="2" max="2" width="56.81640625" customWidth="1"/>
+    <col min="1" max="1" width="24.83203125" customWidth="1"/>
+    <col min="2" max="2" width="56.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="13" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" ht="13" x14ac:dyDescent="0.15">
       <c r="A1" s="1" t="s">
         <v>109</v>
       </c>
       <c r="B1" s="2"/>
     </row>
-    <row r="2" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A2" s="10" t="s">
         <v>3</v>
       </c>
@@ -2236,7 +2419,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="58" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" ht="58" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A3" s="10" t="s">
         <v>110</v>
       </c>
@@ -2244,7 +2427,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="71.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" ht="71.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A4" s="10" t="s">
         <v>111</v>
       </c>
@@ -2252,7 +2435,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="220" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" ht="220" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A5" s="10" t="s">
         <v>113</v>
       </c>
@@ -2260,7 +2443,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="71.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" ht="71.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A6" s="10" t="s">
         <v>115</v>
       </c>
@@ -2268,7 +2451,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="125.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" ht="125.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A7" s="10" t="s">
         <v>117</v>
       </c>
@@ -2276,7 +2459,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A8" s="10" t="s">
         <v>119</v>
       </c>
@@ -2284,7 +2467,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" ht="13" x14ac:dyDescent="0.15">
       <c r="A9" s="10" t="s">
         <v>121</v>
       </c>
@@ -2292,14 +2475,14 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="13" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" ht="13" x14ac:dyDescent="0.15">
       <c r="A11" s="4" t="s">
         <v>109</v>
       </c>
       <c r="B11" s="5"/>
       <c r="C11" s="6"/>
     </row>
-    <row r="12" spans="1:3" ht="112.5" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" ht="126" x14ac:dyDescent="0.15">
       <c r="A12" s="3" t="s">
         <v>122</v>
       </c>
@@ -2307,7 +2490,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" ht="13" x14ac:dyDescent="0.15">
       <c r="A13" s="3" t="s">
         <v>123</v>
       </c>
@@ -2315,7 +2498,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" ht="13" x14ac:dyDescent="0.15">
       <c r="A14" s="3" t="s">
         <v>124</v>
       </c>
@@ -2323,7 +2506,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" ht="13" x14ac:dyDescent="0.15">
       <c r="A15" s="3" t="s">
         <v>125</v>
       </c>
@@ -2331,7 +2514,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" ht="13" x14ac:dyDescent="0.15">
       <c r="A16" s="3" t="s">
         <v>126</v>
       </c>
@@ -2339,14 +2522,66 @@
         <v>46322</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" ht="13" x14ac:dyDescent="0.15">
       <c r="A17" s="3" t="s">
         <v>127</v>
       </c>
-      <c r="B17" s="3" t="inlineStr">
-        <is>
-          <t>6c0c6eb</t>
-        </is>
+      <c r="B17" s="3" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A19" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="B19" s="5"/>
+    </row>
+    <row r="20" spans="1:2" ht="132" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A20" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="B20" s="11" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A21" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A22" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="B22" s="3" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A23" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="B23" s="3" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A24" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="B24" s="12">
+        <v>46323</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A25" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="B25" s="3" t="s">
+        <v>181</v>
       </c>
     </row>
   </sheetData>
@@ -2359,20 +2594,20 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
-  <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:C25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
   <cols>
-    <col min="1" max="1" width="24.81640625" customWidth="1"/>
-    <col min="2" max="2" width="56.81640625" customWidth="1"/>
+    <col min="1" max="1" width="24.83203125" customWidth="1"/>
+    <col min="2" max="2" width="56.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="13" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" ht="13" x14ac:dyDescent="0.15">
       <c r="A1" s="1" t="s">
         <v>109</v>
       </c>
       <c r="B1" s="2"/>
     </row>
-    <row r="2" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A2" s="10" t="s">
         <v>3</v>
       </c>
@@ -2380,7 +2615,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="44.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" ht="44.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A3" s="10" t="s">
         <v>110</v>
       </c>
@@ -2388,7 +2623,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="112" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" ht="112" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A4" s="10" t="s">
         <v>111</v>
       </c>
@@ -2396,7 +2631,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="193" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" ht="193" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A5" s="10" t="s">
         <v>113</v>
       </c>
@@ -2404,7 +2639,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="98.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" ht="98.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A6" s="10" t="s">
         <v>115</v>
       </c>
@@ -2412,7 +2647,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="220" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" ht="220" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A7" s="10" t="s">
         <v>117</v>
       </c>
@@ -2420,7 +2655,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A8" s="10" t="s">
         <v>119</v>
       </c>
@@ -2428,7 +2663,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" ht="13" x14ac:dyDescent="0.15">
       <c r="A9" s="10" t="s">
         <v>121</v>
       </c>
@@ -2436,14 +2671,14 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="13" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" ht="13" x14ac:dyDescent="0.15">
       <c r="A11" s="4" t="s">
         <v>109</v>
       </c>
       <c r="B11" s="5"/>
       <c r="C11" s="6"/>
     </row>
-    <row r="12" spans="1:3" ht="187.5" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" ht="196" x14ac:dyDescent="0.15">
       <c r="A12" s="3" t="s">
         <v>122</v>
       </c>
@@ -2451,7 +2686,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" ht="13" x14ac:dyDescent="0.15">
       <c r="A13" s="3" t="s">
         <v>123</v>
       </c>
@@ -2459,7 +2694,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" ht="13" x14ac:dyDescent="0.15">
       <c r="A14" s="3" t="s">
         <v>124</v>
       </c>
@@ -2467,7 +2702,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" ht="13" x14ac:dyDescent="0.15">
       <c r="A15" s="3" t="s">
         <v>125</v>
       </c>
@@ -2475,7 +2710,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" ht="13" x14ac:dyDescent="0.15">
       <c r="A16" s="3" t="s">
         <v>126</v>
       </c>
@@ -2483,14 +2718,66 @@
         <v>46322</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" ht="13" x14ac:dyDescent="0.15">
       <c r="A17" s="3" t="s">
         <v>127</v>
       </c>
-      <c r="B17" s="3" t="inlineStr">
-        <is>
-          <t>6c0c6eb</t>
-        </is>
+      <c r="B17" s="3" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A19" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="B19" s="5"/>
+    </row>
+    <row r="20" spans="1:2" ht="254" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A20" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="B20" s="11" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A21" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A22" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="B22" s="3" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A23" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="B23" s="3" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A24" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="B24" s="12">
+        <v>46323</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A25" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="B25" s="3" t="s">
+        <v>181</v>
       </c>
     </row>
   </sheetData>
@@ -2503,20 +2790,20 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
-  <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:C25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
   <cols>
-    <col min="1" max="1" width="24.81640625" customWidth="1"/>
-    <col min="2" max="2" width="56.81640625" customWidth="1"/>
+    <col min="1" max="1" width="24.83203125" customWidth="1"/>
+    <col min="2" max="2" width="56.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="13" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" ht="13" x14ac:dyDescent="0.15">
       <c r="A1" s="1" t="s">
         <v>109</v>
       </c>
       <c r="B1" s="2"/>
     </row>
-    <row r="2" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A2" s="10" t="s">
         <v>3</v>
       </c>
@@ -2524,7 +2811,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="44.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" ht="44.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A3" s="10" t="s">
         <v>110</v>
       </c>
@@ -2532,7 +2819,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="71.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" ht="71.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A4" s="10" t="s">
         <v>111</v>
       </c>
@@ -2540,7 +2827,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="166" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" ht="166" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A5" s="10" t="s">
         <v>113</v>
       </c>
@@ -2548,7 +2835,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="58" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" ht="58" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A6" s="10" t="s">
         <v>115</v>
       </c>
@@ -2556,7 +2843,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="301" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" ht="301" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A7" s="10" t="s">
         <v>117</v>
       </c>
@@ -2564,7 +2851,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A8" s="10" t="s">
         <v>119</v>
       </c>
@@ -2572,7 +2859,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" ht="13" x14ac:dyDescent="0.15">
       <c r="A9" s="10" t="s">
         <v>121</v>
       </c>
@@ -2580,14 +2867,14 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="13" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" ht="13" x14ac:dyDescent="0.15">
       <c r="A11" s="4" t="s">
         <v>109</v>
       </c>
       <c r="B11" s="5"/>
       <c r="C11" s="6"/>
     </row>
-    <row r="12" spans="1:3" ht="237.5" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" ht="266" x14ac:dyDescent="0.15">
       <c r="A12" s="3" t="s">
         <v>122</v>
       </c>
@@ -2595,7 +2882,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" ht="13" x14ac:dyDescent="0.15">
       <c r="A13" s="3" t="s">
         <v>123</v>
       </c>
@@ -2603,7 +2890,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" ht="13" x14ac:dyDescent="0.15">
       <c r="A14" s="3" t="s">
         <v>124</v>
       </c>
@@ -2611,7 +2898,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" ht="13" x14ac:dyDescent="0.15">
       <c r="A15" s="3" t="s">
         <v>125</v>
       </c>
@@ -2619,7 +2906,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" ht="13" x14ac:dyDescent="0.15">
       <c r="A16" s="3" t="s">
         <v>126</v>
       </c>
@@ -2627,14 +2914,66 @@
         <v>46322</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" ht="13" x14ac:dyDescent="0.15">
       <c r="A17" s="3" t="s">
         <v>127</v>
       </c>
-      <c r="B17" s="3" t="inlineStr">
-        <is>
-          <t>6c0c6eb</t>
-        </is>
+      <c r="B17" s="3" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A19" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="B19" s="5"/>
+    </row>
+    <row r="20" spans="1:2" ht="279" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A20" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="B20" s="11" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A21" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A22" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="B22" s="3" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A23" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="B23" s="3" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A24" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="B24" s="12">
+        <v>46323</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A25" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="B25" s="3" t="s">
+        <v>181</v>
       </c>
     </row>
   </sheetData>
@@ -2645,14 +2984,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:C17"/>
-  <sheetFormatPr defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="13" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
     <col min="2" max="2" width="75" customWidth="1"/>
     <col min="3" max="3" width="40" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="13" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" ht="14" x14ac:dyDescent="0.15">
       <c r="A1" s="7" t="s">
         <v>90</v>
       </c>
@@ -2663,7 +3002,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="58" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" ht="58" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A2" s="9">
         <v>1</v>
       </c>
@@ -2672,7 +3011,7 @@
       </c>
       <c r="C2" s="9"/>
     </row>
-    <row r="3" spans="1:3" ht="166" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" ht="166" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A3" s="9">
         <v>2</v>
       </c>
@@ -2681,7 +3020,7 @@
       </c>
       <c r="C3" s="9"/>
     </row>
-    <row r="4" spans="1:3" ht="247" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" ht="247" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A4" s="9">
         <v>3</v>
       </c>
@@ -2690,7 +3029,7 @@
       </c>
       <c r="C4" s="9"/>
     </row>
-    <row r="5" spans="1:3" ht="166" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" ht="166" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A5" s="9">
         <v>4</v>
       </c>
@@ -2699,7 +3038,7 @@
       </c>
       <c r="C5" s="9"/>
     </row>
-    <row r="6" spans="1:3" ht="179.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" ht="179.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A6" s="9">
         <v>5</v>
       </c>
@@ -2708,7 +3047,7 @@
       </c>
       <c r="C6" s="9"/>
     </row>
-    <row r="7" spans="1:3" ht="139" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" ht="139" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A7" s="9">
         <v>6</v>
       </c>
@@ -2717,7 +3056,7 @@
       </c>
       <c r="C7" s="9"/>
     </row>
-    <row r="8" spans="1:3" ht="139" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" ht="139" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A8" s="9">
         <v>7</v>
       </c>
@@ -2726,7 +3065,7 @@
       </c>
       <c r="C8" s="9"/>
     </row>
-    <row r="9" spans="1:3" ht="233.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" ht="233.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A9" s="9">
         <v>8</v>
       </c>
@@ -2735,7 +3074,7 @@
       </c>
       <c r="C9" s="9"/>
     </row>
-    <row r="10" spans="1:3" ht="125.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" ht="125.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A10" s="9">
         <v>9</v>
       </c>
@@ -2744,7 +3083,7 @@
       </c>
       <c r="C10" s="9"/>
     </row>
-    <row r="11" spans="1:3" ht="233.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" ht="233.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A11" s="9">
         <v>10</v>
       </c>
@@ -2753,7 +3092,7 @@
       </c>
       <c r="C11" s="9"/>
     </row>
-    <row r="12" spans="1:3" ht="58" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" ht="58" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A12" s="9">
         <v>11</v>
       </c>
@@ -2762,7 +3101,7 @@
       </c>
       <c r="C12" s="9"/>
     </row>
-    <row r="13" spans="1:3" ht="179.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" ht="179.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A13" s="9">
         <v>12</v>
       </c>
@@ -2771,7 +3110,7 @@
       </c>
       <c r="C13" s="9"/>
     </row>
-    <row r="14" spans="1:3" ht="85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" ht="85" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A14" s="9">
         <v>13</v>
       </c>
@@ -2780,7 +3119,7 @@
       </c>
       <c r="C14" s="9"/>
     </row>
-    <row r="15" spans="1:3" ht="98.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" ht="98.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A15" s="9">
         <v>14</v>
       </c>
@@ -2789,7 +3128,7 @@
       </c>
       <c r="C15" s="9"/>
     </row>
-    <row r="16" spans="1:3" ht="71.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" ht="71.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A16" s="9">
         <v>15</v>
       </c>
@@ -2798,7 +3137,7 @@
       </c>
       <c r="C16" s="9"/>
     </row>
-    <row r="17" spans="1:3" ht="382" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:3" ht="382" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A17" s="9">
         <v>16</v>
       </c>
@@ -2817,20 +3156,20 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
-  <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:C26"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
   <cols>
-    <col min="1" max="1" width="24.81640625" customWidth="1"/>
-    <col min="2" max="2" width="56.81640625" customWidth="1"/>
+    <col min="1" max="1" width="24.83203125" customWidth="1"/>
+    <col min="2" max="2" width="56.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="13" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" ht="13" x14ac:dyDescent="0.15">
       <c r="A1" s="1" t="s">
         <v>109</v>
       </c>
       <c r="B1" s="2"/>
     </row>
-    <row r="2" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A2" s="10" t="s">
         <v>3</v>
       </c>
@@ -2838,7 +3177,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="58" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" ht="58" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A3" s="10" t="s">
         <v>110</v>
       </c>
@@ -2846,7 +3185,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="125.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" ht="125.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A4" s="10" t="s">
         <v>111</v>
       </c>
@@ -2854,7 +3193,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="112" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" ht="112" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A5" s="10" t="s">
         <v>113</v>
       </c>
@@ -2862,7 +3201,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="112" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" ht="112" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A6" s="10" t="s">
         <v>115</v>
       </c>
@@ -2870,7 +3209,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="409.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" ht="409.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A7" s="10" t="s">
         <v>117</v>
       </c>
@@ -2878,7 +3217,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A8" s="10" t="s">
         <v>119</v>
       </c>
@@ -2886,7 +3225,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" ht="13" x14ac:dyDescent="0.15">
       <c r="A9" s="10" t="s">
         <v>121</v>
       </c>
@@ -2894,14 +3233,14 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="13" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" ht="13" x14ac:dyDescent="0.15">
       <c r="A11" s="4" t="s">
         <v>109</v>
       </c>
       <c r="B11" s="5"/>
       <c r="C11" s="6"/>
     </row>
-    <row r="12" spans="1:3" ht="387.5" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" ht="409.6" x14ac:dyDescent="0.15">
       <c r="A12" s="3" t="s">
         <v>122</v>
       </c>
@@ -2909,7 +3248,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" ht="13" x14ac:dyDescent="0.15">
       <c r="A13" s="3" t="s">
         <v>123</v>
       </c>
@@ -2917,7 +3256,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" ht="13" x14ac:dyDescent="0.15">
       <c r="A14" s="3" t="s">
         <v>124</v>
       </c>
@@ -2925,7 +3264,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" ht="13" x14ac:dyDescent="0.15">
       <c r="A15" s="3" t="s">
         <v>125</v>
       </c>
@@ -2933,7 +3272,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" ht="13" x14ac:dyDescent="0.15">
       <c r="A16" s="3" t="s">
         <v>126</v>
       </c>
@@ -2941,14 +3280,66 @@
         <v>46322</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" ht="13" x14ac:dyDescent="0.15">
       <c r="A17" s="3" t="s">
         <v>127</v>
       </c>
-      <c r="B17" s="3" t="inlineStr">
-        <is>
-          <t>6c0c6eb</t>
-        </is>
+      <c r="B17" s="3" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A20" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="B20" s="5"/>
+    </row>
+    <row r="21" spans="1:2" ht="370" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A21" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="B21" s="11" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A22" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="B22" s="3" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" ht="16" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A23" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="B23" s="3" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A24" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="B24" s="3" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A25" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="B25" s="12">
+        <v>46323</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A26" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="B26" s="3" t="s">
+        <v>181</v>
       </c>
     </row>
   </sheetData>
@@ -2961,20 +3352,20 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
-  <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:C25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
   <cols>
-    <col min="1" max="1" width="24.81640625" customWidth="1"/>
-    <col min="2" max="2" width="56.81640625" customWidth="1"/>
+    <col min="1" max="1" width="24.83203125" customWidth="1"/>
+    <col min="2" max="2" width="56.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="13" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" ht="13" x14ac:dyDescent="0.15">
       <c r="A1" s="1" t="s">
         <v>109</v>
       </c>
       <c r="B1" s="2"/>
     </row>
-    <row r="2" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A2" s="10" t="s">
         <v>3</v>
       </c>
@@ -2982,7 +3373,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="44.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" ht="44.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A3" s="10" t="s">
         <v>110</v>
       </c>
@@ -2990,7 +3381,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="112" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" ht="112" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A4" s="10" t="s">
         <v>111</v>
       </c>
@@ -2998,7 +3389,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="71.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" ht="71.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A5" s="10" t="s">
         <v>113</v>
       </c>
@@ -3006,7 +3397,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="98.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" ht="98.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A6" s="10" t="s">
         <v>115</v>
       </c>
@@ -3014,7 +3405,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="166" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" ht="166" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A7" s="10" t="s">
         <v>117</v>
       </c>
@@ -3022,7 +3413,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A8" s="10" t="s">
         <v>119</v>
       </c>
@@ -3030,7 +3421,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" ht="13" x14ac:dyDescent="0.15">
       <c r="A9" s="10" t="s">
         <v>121</v>
       </c>
@@ -3038,14 +3429,14 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="13" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" ht="13" x14ac:dyDescent="0.15">
       <c r="A11" s="4" t="s">
         <v>109</v>
       </c>
       <c r="B11" s="5"/>
       <c r="C11" s="6"/>
     </row>
-    <row r="12" spans="1:3" ht="125" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" ht="140" x14ac:dyDescent="0.15">
       <c r="A12" s="3" t="s">
         <v>122</v>
       </c>
@@ -3053,7 +3444,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" ht="13" x14ac:dyDescent="0.15">
       <c r="A13" s="3" t="s">
         <v>123</v>
       </c>
@@ -3061,7 +3452,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" ht="13" x14ac:dyDescent="0.15">
       <c r="A14" s="3" t="s">
         <v>124</v>
       </c>
@@ -3069,7 +3460,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" ht="13" x14ac:dyDescent="0.15">
       <c r="A15" s="3" t="s">
         <v>125</v>
       </c>
@@ -3077,7 +3468,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" ht="13" x14ac:dyDescent="0.15">
       <c r="A16" s="3" t="s">
         <v>126</v>
       </c>
@@ -3085,14 +3476,69 @@
         <v>46322</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" ht="13" x14ac:dyDescent="0.15">
       <c r="A17" s="3" t="s">
         <v>127</v>
       </c>
-      <c r="B17" s="3" t="inlineStr">
+      <c r="B17" s="3" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A19" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="B19" s="5"/>
+    </row>
+    <row r="20" spans="1:2" ht="174" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A20" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="B20" s="11" t="inlineStr">
         <is>
-          <t>6c0c6eb</t>
+          <t>Step 4: Exactly one card matches: 'SPM38 Guarded Forum', 'SPM38 Studio (SPM38-STU)', with the 'Pending' badge, 'Requested' '9 Feb 2028, 09:00–12:00', and its 'Approve' and 'Reject with a reason' buttons. No card for 'SPM38 Lantern Gala' is on the page.
+Step 5: The Notifications list has a new notification titled 'Venue booking released' for 'SPM38 Lantern Gala', reading 'Daniel Tan released SPM38 Hall (SPM38-HAL) for EVT-002670 SPM38 Lantern Gala on 12 Jan 2028, 09:00–12:00. Reason: Event postponed: The client is waiting on board approval before choosing a new date.' There is no notification about the withdrawn SPM38 Studio request.</t>
         </is>
+      </c>
+    </row>
+    <row r="21" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A21" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A22" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="B22" s="3" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A23" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="B23" s="3" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A24" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="B24" s="12">
+        <v>46323</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A25" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="B25" s="3" t="s">
+        <v>181</v>
       </c>
     </row>
   </sheetData>
@@ -3105,20 +3551,20 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
-  <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:C25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
   <cols>
-    <col min="1" max="1" width="24.81640625" customWidth="1"/>
-    <col min="2" max="2" width="56.81640625" customWidth="1"/>
+    <col min="1" max="1" width="24.83203125" customWidth="1"/>
+    <col min="2" max="2" width="56.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="13" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" ht="13" x14ac:dyDescent="0.15">
       <c r="A1" s="1" t="s">
         <v>109</v>
       </c>
       <c r="B1" s="2"/>
     </row>
-    <row r="2" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A2" s="10" t="s">
         <v>3</v>
       </c>
@@ -3126,7 +3572,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="31" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" ht="31" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A3" s="10" t="s">
         <v>110</v>
       </c>
@@ -3134,7 +3580,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="139" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" ht="139" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A4" s="10" t="s">
         <v>111</v>
       </c>
@@ -3142,7 +3588,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="287.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" ht="287.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A5" s="10" t="s">
         <v>113</v>
       </c>
@@ -3150,7 +3596,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" ht="85" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A6" s="10" t="s">
         <v>115</v>
       </c>
@@ -3158,7 +3604,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="274" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" ht="274" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A7" s="10" t="s">
         <v>117</v>
       </c>
@@ -3166,7 +3612,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A8" s="10" t="s">
         <v>119</v>
       </c>
@@ -3174,7 +3620,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" ht="13" x14ac:dyDescent="0.15">
       <c r="A9" s="10" t="s">
         <v>121</v>
       </c>
@@ -3182,14 +3628,14 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="13" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" ht="13" x14ac:dyDescent="0.15">
       <c r="A11" s="4" t="s">
         <v>109</v>
       </c>
       <c r="B11" s="5"/>
       <c r="C11" s="6"/>
     </row>
-    <row r="12" spans="1:3" ht="212.5" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" ht="238" x14ac:dyDescent="0.15">
       <c r="A12" s="3" t="s">
         <v>122</v>
       </c>
@@ -3197,7 +3643,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" ht="13" x14ac:dyDescent="0.15">
       <c r="A13" s="3" t="s">
         <v>123</v>
       </c>
@@ -3205,7 +3651,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" ht="13" x14ac:dyDescent="0.15">
       <c r="A14" s="3" t="s">
         <v>124</v>
       </c>
@@ -3213,7 +3659,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" ht="13" x14ac:dyDescent="0.15">
       <c r="A15" s="3" t="s">
         <v>125</v>
       </c>
@@ -3221,7 +3667,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" ht="13" x14ac:dyDescent="0.15">
       <c r="A16" s="3" t="s">
         <v>126</v>
       </c>
@@ -3229,14 +3675,74 @@
         <v>46322</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" ht="13" x14ac:dyDescent="0.15">
       <c r="A17" s="3" t="s">
         <v>127</v>
       </c>
-      <c r="B17" s="3" t="inlineStr">
+      <c r="B17" s="3" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A19" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="B19" s="5"/>
+    </row>
+    <row r="20" spans="1:2" ht="247" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A20" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="B20" s="11" t="inlineStr">
         <is>
-          <t>6c0c6eb</t>
+          <t>Step 2: The 'SPM38 Projector' line reads '2 total − 0 out of service − 2 reserved elsewhere = 0 available for these dates' and 'Held by SPM38 Riverside Expo (2 units) until 20 Jan.'
+Step 6: The 'Request a venue booking' form opens for SPM38 Hall, with 'Date' 19 Jan 2028, 'Start time' 09:00 and 'End time' 12:00.
+Step 7: The request is not sent. A red alert reads 'SPM38 Hall is already booked for EVT-002671 SPM38 Riverside Expo on 19 Jan 2028, 09:00–12:00.'
+Step 9: The dialog 'Postpone this event?' lists 'Release SPM38 Hall (SPM38-HAL) on 19 Jan 2028, 09:00–12:00' and 'Release 2 × SPM38 Projector'.
+Step 10: The badge reads 'Postponed'.
+Step 13: A green alert reads 'Booking request sent to Venue Staff.' The postponed event's booking no longer blocks the Hall.
+Step 16: The 'SPM38 Projector' line reads '2 total − 0 out of service − 0 reserved elsewhere = 2 available for these dates', with no 'Held by' line.</t>
         </is>
+      </c>
+    </row>
+    <row r="21" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A21" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A22" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="B22" s="3" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A23" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="B23" s="3" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A24" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="B24" s="12">
+        <v>46323</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A25" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="B25" s="3" t="s">
+        <v>181</v>
       </c>
     </row>
   </sheetData>
@@ -3249,20 +3755,20 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
-  <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:C25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
   <cols>
-    <col min="1" max="1" width="24.81640625" customWidth="1"/>
-    <col min="2" max="2" width="56.81640625" customWidth="1"/>
+    <col min="1" max="1" width="24.83203125" customWidth="1"/>
+    <col min="2" max="2" width="56.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="13" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" ht="13" x14ac:dyDescent="0.15">
       <c r="A1" s="1" t="s">
         <v>109</v>
       </c>
       <c r="B1" s="2"/>
     </row>
-    <row r="2" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A2" s="10" t="s">
         <v>3</v>
       </c>
@@ -3270,7 +3776,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="31" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" ht="31" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A3" s="10" t="s">
         <v>110</v>
       </c>
@@ -3278,7 +3784,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="98.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" ht="98.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A4" s="10" t="s">
         <v>111</v>
       </c>
@@ -3286,7 +3792,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="179.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" ht="179.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A5" s="10" t="s">
         <v>113</v>
       </c>
@@ -3294,7 +3800,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="44.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" ht="44.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A6" s="10" t="s">
         <v>115</v>
       </c>
@@ -3302,7 +3808,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="152.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" ht="152.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A7" s="10" t="s">
         <v>117</v>
       </c>
@@ -3310,7 +3816,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A8" s="10" t="s">
         <v>119</v>
       </c>
@@ -3318,7 +3824,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" ht="13" x14ac:dyDescent="0.15">
       <c r="A9" s="10" t="s">
         <v>121</v>
       </c>
@@ -3326,14 +3832,14 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="13" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" ht="13" x14ac:dyDescent="0.15">
       <c r="A11" s="4" t="s">
         <v>109</v>
       </c>
       <c r="B11" s="5"/>
       <c r="C11" s="6"/>
     </row>
-    <row r="12" spans="1:3" ht="125" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" ht="140" x14ac:dyDescent="0.15">
       <c r="A12" s="3" t="s">
         <v>122</v>
       </c>
@@ -3341,7 +3847,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" ht="13" x14ac:dyDescent="0.15">
       <c r="A13" s="3" t="s">
         <v>123</v>
       </c>
@@ -3349,7 +3855,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" ht="13" x14ac:dyDescent="0.15">
       <c r="A14" s="3" t="s">
         <v>124</v>
       </c>
@@ -3357,7 +3863,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" ht="13" x14ac:dyDescent="0.15">
       <c r="A15" s="3" t="s">
         <v>125</v>
       </c>
@@ -3365,7 +3871,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" ht="13" x14ac:dyDescent="0.15">
       <c r="A16" s="3" t="s">
         <v>126</v>
       </c>
@@ -3373,14 +3879,66 @@
         <v>46322</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" ht="13" x14ac:dyDescent="0.15">
       <c r="A17" s="3" t="s">
         <v>127</v>
       </c>
-      <c r="B17" s="3" t="inlineStr">
-        <is>
-          <t>6c0c6eb</t>
-        </is>
+      <c r="B17" s="3" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A19" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="B19" s="5"/>
+    </row>
+    <row r="20" spans="1:2" ht="146" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A20" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="B20" s="11" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A21" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A22" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="B22" s="3" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A23" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="B23" s="3" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A24" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="B24" s="12">
+        <v>46323</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A25" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="B25" s="3" t="s">
+        <v>181</v>
       </c>
     </row>
   </sheetData>
@@ -3393,20 +3951,20 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
-  <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:C25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
   <cols>
-    <col min="1" max="1" width="24.81640625" customWidth="1"/>
-    <col min="2" max="2" width="56.81640625" customWidth="1"/>
+    <col min="1" max="1" width="24.83203125" customWidth="1"/>
+    <col min="2" max="2" width="56.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="13" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" ht="13" x14ac:dyDescent="0.15">
       <c r="A1" s="1" t="s">
         <v>109</v>
       </c>
       <c r="B1" s="2"/>
     </row>
-    <row r="2" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A2" s="10" t="s">
         <v>3</v>
       </c>
@@ -3414,7 +3972,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="44.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" ht="44.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A3" s="10" t="s">
         <v>110</v>
       </c>
@@ -3422,7 +3980,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" ht="85" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A4" s="10" t="s">
         <v>111</v>
       </c>
@@ -3430,7 +3988,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="112" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" ht="112" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A5" s="10" t="s">
         <v>113</v>
       </c>
@@ -3438,7 +3996,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="58" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" ht="58" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A6" s="10" t="s">
         <v>115</v>
       </c>
@@ -3446,7 +4004,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="152.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" ht="152.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A7" s="10" t="s">
         <v>117</v>
       </c>
@@ -3454,7 +4012,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A8" s="10" t="s">
         <v>119</v>
       </c>
@@ -3462,7 +4020,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" ht="13" x14ac:dyDescent="0.15">
       <c r="A9" s="10" t="s">
         <v>121</v>
       </c>
@@ -3470,14 +4028,14 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="13" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" ht="13" x14ac:dyDescent="0.15">
       <c r="A11" s="4" t="s">
         <v>109</v>
       </c>
       <c r="B11" s="5"/>
       <c r="C11" s="6"/>
     </row>
-    <row r="12" spans="1:3" ht="137.5" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" ht="154" x14ac:dyDescent="0.15">
       <c r="A12" s="3" t="s">
         <v>122</v>
       </c>
@@ -3485,7 +4043,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" ht="13" x14ac:dyDescent="0.15">
       <c r="A13" s="3" t="s">
         <v>123</v>
       </c>
@@ -3493,7 +4051,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" ht="13" x14ac:dyDescent="0.15">
       <c r="A14" s="3" t="s">
         <v>124</v>
       </c>
@@ -3501,7 +4059,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" ht="13" x14ac:dyDescent="0.15">
       <c r="A15" s="3" t="s">
         <v>125</v>
       </c>
@@ -3509,7 +4067,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" ht="13" x14ac:dyDescent="0.15">
       <c r="A16" s="3" t="s">
         <v>126</v>
       </c>
@@ -3517,14 +4075,66 @@
         <v>46322</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" ht="13" x14ac:dyDescent="0.15">
       <c r="A17" s="3" t="s">
         <v>127</v>
       </c>
-      <c r="B17" s="3" t="inlineStr">
-        <is>
-          <t>6c0c6eb</t>
-        </is>
+      <c r="B17" s="3" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A19" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="B19" s="5"/>
+    </row>
+    <row r="20" spans="1:2" ht="189" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A20" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="B20" s="11" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A21" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A22" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="B22" s="3" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A23" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="B23" s="3" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A24" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="B24" s="12">
+        <v>46323</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A25" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="B25" s="3" t="s">
+        <v>181</v>
       </c>
     </row>
   </sheetData>
@@ -3537,20 +4147,20 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
-  <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:C25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
   <cols>
-    <col min="1" max="1" width="24.81640625" customWidth="1"/>
-    <col min="2" max="2" width="56.81640625" customWidth="1"/>
+    <col min="1" max="1" width="24.83203125" customWidth="1"/>
+    <col min="2" max="2" width="56.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="13" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" ht="13" x14ac:dyDescent="0.15">
       <c r="A1" s="1" t="s">
         <v>109</v>
       </c>
       <c r="B1" s="2"/>
     </row>
-    <row r="2" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A2" s="10" t="s">
         <v>3</v>
       </c>
@@ -3558,7 +4168,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="44.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" ht="44.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A3" s="10" t="s">
         <v>110</v>
       </c>
@@ -3566,7 +4176,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="125.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" ht="125.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A4" s="10" t="s">
         <v>111</v>
       </c>
@@ -3574,7 +4184,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="139" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" ht="139" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A5" s="10" t="s">
         <v>113</v>
       </c>
@@ -3582,7 +4192,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="98.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" ht="98.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A6" s="10" t="s">
         <v>115</v>
       </c>
@@ -3590,7 +4200,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="206.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" ht="206.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A7" s="10" t="s">
         <v>117</v>
       </c>
@@ -3598,7 +4208,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A8" s="10" t="s">
         <v>119</v>
       </c>
@@ -3606,7 +4216,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" ht="13" x14ac:dyDescent="0.15">
       <c r="A9" s="10" t="s">
         <v>121</v>
       </c>
@@ -3614,14 +4224,14 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="13" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" ht="13" x14ac:dyDescent="0.15">
       <c r="A11" s="4" t="s">
         <v>109</v>
       </c>
       <c r="B11" s="5"/>
       <c r="C11" s="6"/>
     </row>
-    <row r="12" spans="1:3" ht="175" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" ht="196" x14ac:dyDescent="0.15">
       <c r="A12" s="3" t="s">
         <v>122</v>
       </c>
@@ -3629,7 +4239,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" ht="13" x14ac:dyDescent="0.15">
       <c r="A13" s="3" t="s">
         <v>123</v>
       </c>
@@ -3637,7 +4247,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" ht="13" x14ac:dyDescent="0.15">
       <c r="A14" s="3" t="s">
         <v>124</v>
       </c>
@@ -3645,7 +4255,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" ht="13" x14ac:dyDescent="0.15">
       <c r="A15" s="3" t="s">
         <v>125</v>
       </c>
@@ -3653,7 +4263,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" ht="13" x14ac:dyDescent="0.15">
       <c r="A16" s="3" t="s">
         <v>126</v>
       </c>
@@ -3661,14 +4271,66 @@
         <v>46322</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" ht="13" x14ac:dyDescent="0.15">
       <c r="A17" s="3" t="s">
         <v>127</v>
       </c>
-      <c r="B17" s="3" t="inlineStr">
-        <is>
-          <t>6c0c6eb</t>
-        </is>
+      <c r="B17" s="3" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A19" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="B19" s="5"/>
+    </row>
+    <row r="20" spans="1:2" ht="206" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A20" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="B20" s="11" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A21" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A22" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="B22" s="3" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A23" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="B23" s="3" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A24" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="B24" s="12">
+        <v>46323</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A25" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="B25" s="3" t="s">
+        <v>181</v>
       </c>
     </row>
   </sheetData>
@@ -3681,20 +4343,20 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
-  <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:C26"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
   <cols>
-    <col min="1" max="1" width="24.81640625" customWidth="1"/>
-    <col min="2" max="2" width="56.81640625" customWidth="1"/>
+    <col min="1" max="1" width="24.83203125" customWidth="1"/>
+    <col min="2" max="2" width="56.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="13" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" ht="13" x14ac:dyDescent="0.15">
       <c r="A1" s="1" t="s">
         <v>109</v>
       </c>
       <c r="B1" s="2"/>
     </row>
-    <row r="2" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A2" s="10" t="s">
         <v>3</v>
       </c>
@@ -3702,7 +4364,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="58" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" ht="58" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A3" s="10" t="s">
         <v>110</v>
       </c>
@@ -3710,7 +4372,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="112" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" ht="112" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A4" s="10" t="s">
         <v>111</v>
       </c>
@@ -3718,7 +4380,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="260.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" ht="260.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A5" s="10" t="s">
         <v>113</v>
       </c>
@@ -3726,7 +4388,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" ht="85" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A6" s="10" t="s">
         <v>115</v>
       </c>
@@ -3734,7 +4396,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="193" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" ht="193" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A7" s="10" t="s">
         <v>117</v>
       </c>
@@ -3742,7 +4404,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A8" s="10" t="s">
         <v>119</v>
       </c>
@@ -3750,7 +4412,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" ht="13" x14ac:dyDescent="0.15">
       <c r="A9" s="10" t="s">
         <v>121</v>
       </c>
@@ -3758,14 +4420,14 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="13" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" ht="13" x14ac:dyDescent="0.15">
       <c r="A11" s="4" t="s">
         <v>109</v>
       </c>
       <c r="B11" s="5"/>
       <c r="C11" s="6"/>
     </row>
-    <row r="12" spans="1:3" ht="150" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" ht="168" x14ac:dyDescent="0.15">
       <c r="A12" s="3" t="s">
         <v>122</v>
       </c>
@@ -3773,7 +4435,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" ht="13" x14ac:dyDescent="0.15">
       <c r="A13" s="3" t="s">
         <v>123</v>
       </c>
@@ -3781,7 +4443,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" ht="13" x14ac:dyDescent="0.15">
       <c r="A14" s="3" t="s">
         <v>124</v>
       </c>
@@ -3789,7 +4451,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" ht="13" x14ac:dyDescent="0.15">
       <c r="A15" s="3" t="s">
         <v>125</v>
       </c>
@@ -3797,7 +4459,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" ht="13" x14ac:dyDescent="0.15">
       <c r="A16" s="3" t="s">
         <v>126</v>
       </c>
@@ -3805,14 +4467,66 @@
         <v>46322</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" ht="13" x14ac:dyDescent="0.15">
       <c r="A17" s="3" t="s">
         <v>127</v>
       </c>
-      <c r="B17" s="3" t="inlineStr">
-        <is>
-          <t>6c0c6eb</t>
-        </is>
+      <c r="B17" s="3" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A20" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="B20" s="5"/>
+    </row>
+    <row r="21" spans="1:2" ht="209" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A21" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="B21" s="11" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A22" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="B22" s="3" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A23" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="B23" s="3" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A24" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="B24" s="3" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A25" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="B25" s="12">
+        <v>46323</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A26" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="B26" s="3" t="s">
+        <v>181</v>
       </c>
     </row>
   </sheetData>

</xml_diff>